<commit_message>
feat: remove valuations feature from entire codebase
Valuations (monthly billing periods) were dormant infrastructure — never
displayed on the website, adding mandatory friction to cost and AR invoice
entry. Removed the table, all references, CLI module, import templates,
and documentation.

- Migration drops valuations table, FK constraints, indexes, columns, RLS
- CLI: delete valuations.py, remove from costs.py/ar_invoices.py/main.py
- Import: remove valuation template and lookup/validation helpers
- Website: remove Valuation type (database.types.ts regen pending)
- Docs: clean all 7 numbered docs, skills, CLAUDE.md, TODO.md

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/imports/templates/ar_invoices.xlsx
+++ b/imports/templates/ar_invoices.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U4"/>
+  <dimension ref="A1:T4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -492,13 +492,12 @@
     <col width="44" customWidth="1" min="12" max="12"/>
     <col width="44" customWidth="1" min="13" max="13"/>
     <col width="44" customWidth="1" min="14" max="14"/>
-    <col width="44" customWidth="1" min="15" max="15"/>
-    <col width="38" customWidth="1" min="16" max="16"/>
+    <col width="38" customWidth="1" min="15" max="15"/>
+    <col width="44" customWidth="1" min="16" max="16"/>
     <col width="44" customWidth="1" min="17" max="17"/>
     <col width="44" customWidth="1" min="18" max="18"/>
     <col width="44" customWidth="1" min="19" max="19"/>
-    <col width="44" customWidth="1" min="20" max="20"/>
-    <col width="32" customWidth="1" min="21" max="21"/>
+    <col width="30" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -509,100 +508,95 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>valuation_number</t>
+          <t>bank_name</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>bank_name</t>
+          <t>bank_account_last4</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>bank_account_last4</t>
+          <t>entity_document_number</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>entity_document_number</t>
+          <t>partner_company_name</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>partner_company_name</t>
+          <t>invoice_number</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>invoice_number</t>
+          <t>comprobante_type</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>comprobante_type</t>
+          <t>invoice_date</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>invoice_date</t>
+          <t>due_date</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>due_date</t>
+          <t>subtotal</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>subtotal</t>
+          <t>igv_rate</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>igv_rate</t>
+          <t>detraccion_rate</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>detraccion_rate</t>
+          <t>retencion_applicable</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>retencion_applicable</t>
+          <t>retencion_rate</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>retencion_rate</t>
+          <t>currency</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>currency</t>
+          <t>exchange_rate</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
-          <t>exchange_rate</t>
+          <t>document_ref</t>
         </is>
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
-          <t>document_ref</t>
+          <t>is_internal_settlement</t>
         </is>
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
-          <t>is_internal_settlement</t>
+          <t>retencion_verified</t>
         </is>
       </c>
       <c r="T1" s="1" t="inlineStr">
-        <is>
-          <t>retencion_verified</t>
-        </is>
-      </c>
-      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
@@ -616,89 +610,89 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Interbank</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Interbank</t>
+          <t>7890</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>7890</t>
+          <t>20198765432</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>20198765432</t>
+          <t>Korakuen Ingeniería S.A.C.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Korakuen Ingeniería S.A.C.</t>
+          <t>F001-00089</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>F001-00089</t>
+          <t>factura</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>factura</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>150000.00</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>150000.00</t>
+          <t>18</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>4</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>false</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="P2" s="2" t="inlineStr">
+        <is>
+          <t>3.72</t>
+        </is>
+      </c>
+      <c r="Q2" s="2" t="inlineStr">
+        <is>
+          <t>PRY001-AR-001</t>
+        </is>
+      </c>
+      <c r="R2" s="2" t="inlineStr">
+        <is>
           <t>false</t>
         </is>
       </c>
-      <c r="O2" s="2" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="P2" s="2" t="inlineStr">
-        <is>
-          <t>PEN</t>
-        </is>
-      </c>
-      <c r="Q2" s="2" t="inlineStr">
-        <is>
-          <t>3.72</t>
-        </is>
-      </c>
-      <c r="R2" s="2" t="inlineStr">
-        <is>
-          <t>PRY001-AR-001</t>
-        </is>
-      </c>
       <c r="S2" s="2" t="inlineStr">
         <is>
           <t>false</t>
@@ -706,12 +700,7 @@
       </c>
       <c r="T2" s="2" t="inlineStr">
         <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="U2" s="2" t="inlineStr">
-        <is>
-          <t>March 2026 valuation billing</t>
+          <t>March 2026 billing</t>
         </is>
       </c>
     </row>
@@ -723,100 +712,95 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Required. Valuation number within the project. Must exist.</t>
+          <t>Required. Bank name of the receipt account. Used with bank_account_last4.</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Required. Bank name of the receipt account. Used with bank_account_last4.</t>
+          <t>Required. Last 4 digits of receipt bank account.</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Required. Last 4 digits of receipt bank account.</t>
+          <t>Required. Document number of the client entity.</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Required. Document number of the client entity.</t>
+          <t>Required. Name of the partner company that issued the invoice.</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Required. Name of the partner company that issued the invoice.</t>
+          <t>Required. Own invoice numbering from Alegra/Contasis.</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>Required. Own invoice numbering from Alegra/Contasis.</t>
+          <t>Required. Type of payment document. Always factura for construction AR.</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>Required. Type of payment document. Always factura for construction AR.</t>
+          <t>Required. Invoice issue date. Format: YYYY-MM-DD.</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>Required. Invoice issue date. Format: YYYY-MM-DD.</t>
+          <t>Optional. Payment due date. Format: YYYY-MM-DD.</t>
         </is>
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>Optional. Payment due date. Format: YYYY-MM-DD.</t>
+          <t>Required. NUMERIC(15,2). Invoice subtotal amount.</t>
         </is>
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>Required. NUMERIC(15,2). Entered directly from valuation billed value.</t>
+          <t>Required. IGV percentage. NUMERIC(5,2). Default 18.</t>
         </is>
       </c>
       <c r="L3" s="3" t="inlineStr">
         <is>
-          <t>Required. IGV percentage. NUMERIC(5,2). Default 18.</t>
+          <t>Optional. Detracción percentage. NUMERIC(5,2). Null if not applicable.</t>
         </is>
       </c>
       <c r="M3" s="3" t="inlineStr">
         <is>
-          <t>Optional. Detracción percentage. NUMERIC(5,2). Null if not applicable.</t>
+          <t>Required. Whether client will withhold retención. BOOLEAN.</t>
         </is>
       </c>
       <c r="N3" s="3" t="inlineStr">
         <is>
-          <t>Required. Whether client will withhold retención. BOOLEAN.</t>
+          <t>Optional. Retención percentage. NUMERIC(5,2). Required if retencion_applicable is true. Default 3.</t>
         </is>
       </c>
       <c r="O3" s="3" t="inlineStr">
         <is>
-          <t>Optional. Retención percentage. NUMERIC(5,2). Required if retencion_applicable is true. Default 3.</t>
+          <t>Required. Currency of the invoice.</t>
         </is>
       </c>
       <c r="P3" s="3" t="inlineStr">
         <is>
-          <t>Required. Currency of the invoice.</t>
+          <t>Required. PEN per USD rate at transaction date. NUMERIC(10,4).</t>
         </is>
       </c>
       <c r="Q3" s="3" t="inlineStr">
         <is>
-          <t>Required. PEN per USD rate at transaction date. NUMERIC(10,4).</t>
+          <t>Optional. Document reference linking to SharePoint file.</t>
         </is>
       </c>
       <c r="R3" s="3" t="inlineStr">
         <is>
-          <t>Optional. Document reference linking to SharePoint file.</t>
+          <t>Required. True when invoicing a partner company for settlement. BOOLEAN. Default false.</t>
         </is>
       </c>
       <c r="S3" s="3" t="inlineStr">
         <is>
-          <t>Required. True when invoicing a partner company for settlement. BOOLEAN. Default false.</t>
+          <t>Required. Manually set to true once confirmed that client paid retención to SUNAT. BOOLEAN. Default false.</t>
         </is>
       </c>
       <c r="T3" s="3" t="inlineStr">
-        <is>
-          <t>Required. Manually set to true once confirmed that client paid retención to SUNAT. BOOLEAN. Default false.</t>
-        </is>
-      </c>
-      <c r="U3" s="3" t="inlineStr">
         <is>
           <t>Optional. Free text notes.</t>
         </is>
@@ -830,76 +814,71 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Lookup → valuations (by project + number)</t>
+          <t>Lookup → bank_accounts.bank_name</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Lookup → bank_accounts.bank_name</t>
+          <t>Lookup → bank_accounts.account_number_last4</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Lookup → bank_accounts.account_number_last4</t>
+          <t>Lookup → entities.document_number</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Lookup → entities.document_number</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
           <t>Lookup → partner_companies.name</t>
         </is>
       </c>
-      <c r="G4" s="4" t="inlineStr"/>
-      <c r="H4" s="4" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr"/>
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>factura | boleta | recibo_por_honorarios</t>
         </is>
       </c>
+      <c r="H4" s="4" t="inlineStr"/>
       <c r="I4" s="4" t="inlineStr"/>
       <c r="J4" s="4" t="inlineStr"/>
-      <c r="K4" s="4" t="inlineStr"/>
+      <c r="K4" s="4" t="inlineStr">
+        <is>
+          <t>Usually 18</t>
+        </is>
+      </c>
       <c r="L4" s="4" t="inlineStr">
         <is>
-          <t>Usually 18</t>
+          <t>Varies by service type</t>
         </is>
       </c>
       <c r="M4" s="4" t="inlineStr">
         <is>
-          <t>Varies by service type</t>
+          <t>true | false</t>
         </is>
       </c>
       <c r="N4" s="4" t="inlineStr">
         <is>
+          <t>Usually 3 (if applicable)</t>
+        </is>
+      </c>
+      <c r="O4" s="4" t="inlineStr">
+        <is>
+          <t>USD | PEN</t>
+        </is>
+      </c>
+      <c r="P4" s="4" t="inlineStr"/>
+      <c r="Q4" s="4" t="inlineStr"/>
+      <c r="R4" s="4" t="inlineStr">
+        <is>
           <t>true | false</t>
         </is>
       </c>
-      <c r="O4" s="4" t="inlineStr">
-        <is>
-          <t>Usually 3 (if applicable)</t>
-        </is>
-      </c>
-      <c r="P4" s="4" t="inlineStr">
-        <is>
-          <t>USD | PEN</t>
-        </is>
-      </c>
-      <c r="Q4" s="4" t="inlineStr"/>
-      <c r="R4" s="4" t="inlineStr"/>
       <c r="S4" s="4" t="inlineStr">
         <is>
           <t>true | false</t>
         </is>
       </c>
-      <c r="T4" s="4" t="inlineStr">
-        <is>
-          <t>true | false</t>
-        </is>
-      </c>
-      <c r="U4" s="4" t="inlineStr"/>
+      <c r="T4" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat: combined cost import template + bank account labels
Replace two-step cost import (headers then items) with single atomic
template. Each row is a cost item; rows grouped by document_ref form
one cost with multiple items. Derives cost_type from project_code,
auto-looks up exchange_rate by date from exchange_rates table.

Add label column to bank_accounts for single-field import lookups,
replacing the bank_name + last4 composite key across all templates.
Fix fn_create_cost_with_items RPC to remove dropped valuation_id.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/imports/templates/ar_invoices.xlsx
+++ b/imports/templates/ar_invoices.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T4"/>
+  <dimension ref="A1:R4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -491,13 +491,11 @@
     <col width="44" customWidth="1" min="11" max="11"/>
     <col width="44" customWidth="1" min="12" max="12"/>
     <col width="44" customWidth="1" min="13" max="13"/>
-    <col width="44" customWidth="1" min="14" max="14"/>
-    <col width="38" customWidth="1" min="15" max="15"/>
+    <col width="38" customWidth="1" min="14" max="14"/>
+    <col width="44" customWidth="1" min="15" max="15"/>
     <col width="44" customWidth="1" min="16" max="16"/>
     <col width="44" customWidth="1" min="17" max="17"/>
-    <col width="44" customWidth="1" min="18" max="18"/>
-    <col width="44" customWidth="1" min="19" max="19"/>
-    <col width="30" customWidth="1" min="20" max="20"/>
+    <col width="30" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -508,95 +506,85 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>bank_name</t>
+          <t>bank_account</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>bank_account_last4</t>
+          <t>entity_document_number</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>entity_document_number</t>
+          <t>partner_company_name</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>partner_company_name</t>
+          <t>invoice_number</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>invoice_number</t>
+          <t>comprobante_type</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>comprobante_type</t>
+          <t>invoice_date</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>invoice_date</t>
+          <t>due_date</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>due_date</t>
+          <t>subtotal</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>subtotal</t>
+          <t>igv_rate</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>igv_rate</t>
+          <t>detraccion_rate</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>detraccion_rate</t>
+          <t>retencion_applicable</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>retencion_applicable</t>
+          <t>retencion_rate</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>retencion_rate</t>
+          <t>currency</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>currency</t>
+          <t>exchange_rate</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>exchange_rate</t>
+          <t>document_ref</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
-          <t>document_ref</t>
+          <t>retencion_verified</t>
         </is>
       </c>
       <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>is_internal_settlement</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>retencion_verified</t>
-        </is>
-      </c>
-      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
@@ -610,95 +598,85 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Interbank</t>
+          <t>Interbank-7890</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>7890</t>
+          <t>20198765432</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>20198765432</t>
+          <t>Korakuen Ingeniería S.A.C.</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Korakuen Ingeniería S.A.C.</t>
+          <t>F001-00089</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>F001-00089</t>
+          <t>factura</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>factura</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>150000.00</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>150000.00</t>
+          <t>18</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>4</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>false</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>3.72</t>
+        </is>
+      </c>
+      <c r="P2" s="2" t="inlineStr">
+        <is>
+          <t>PRY001-AR-001</t>
+        </is>
+      </c>
+      <c r="Q2" s="2" t="inlineStr">
+        <is>
           <t>false</t>
         </is>
       </c>
-      <c r="N2" s="2" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="O2" s="2" t="inlineStr">
-        <is>
-          <t>PEN</t>
-        </is>
-      </c>
-      <c r="P2" s="2" t="inlineStr">
-        <is>
-          <t>3.72</t>
-        </is>
-      </c>
-      <c r="Q2" s="2" t="inlineStr">
-        <is>
-          <t>PRY001-AR-001</t>
-        </is>
-      </c>
       <c r="R2" s="2" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="S2" s="2" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="T2" s="2" t="inlineStr">
         <is>
           <t>March 2026 billing</t>
         </is>
@@ -712,95 +690,85 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Required. Bank name of the receipt account. Used with bank_account_last4.</t>
+          <t>Required. Bank account label. Must exist in bank_accounts table.</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Required. Last 4 digits of receipt bank account.</t>
+          <t>Required. Document number of the client entity.</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Required. Document number of the client entity.</t>
+          <t>Required. Name of the partner company that issued the invoice.</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Required. Name of the partner company that issued the invoice.</t>
+          <t>Required. Own invoice numbering from Alegra/Contasis.</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Required. Own invoice numbering from Alegra/Contasis.</t>
+          <t>Required. Type of payment document. Always factura for construction AR.</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>Required. Type of payment document. Always factura for construction AR.</t>
+          <t>Required. Invoice issue date. Format: YYYY-MM-DD.</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>Required. Invoice issue date. Format: YYYY-MM-DD.</t>
+          <t>Optional. Payment due date. Format: YYYY-MM-DD.</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>Optional. Payment due date. Format: YYYY-MM-DD.</t>
+          <t>Required. NUMERIC(15,2). Invoice subtotal amount.</t>
         </is>
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>Required. NUMERIC(15,2). Invoice subtotal amount.</t>
+          <t>Required. IGV percentage. NUMERIC(5,2). Default 18.</t>
         </is>
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>Required. IGV percentage. NUMERIC(5,2). Default 18.</t>
+          <t>Optional. Detracción percentage. NUMERIC(5,2). Null if not applicable.</t>
         </is>
       </c>
       <c r="L3" s="3" t="inlineStr">
         <is>
-          <t>Optional. Detracción percentage. NUMERIC(5,2). Null if not applicable.</t>
+          <t>Required. Whether client will withhold retención. BOOLEAN.</t>
         </is>
       </c>
       <c r="M3" s="3" t="inlineStr">
         <is>
-          <t>Required. Whether client will withhold retención. BOOLEAN.</t>
+          <t>Optional. Retención percentage. NUMERIC(5,2). Required if retencion_applicable is true. Default 3.</t>
         </is>
       </c>
       <c r="N3" s="3" t="inlineStr">
         <is>
-          <t>Optional. Retención percentage. NUMERIC(5,2). Required if retencion_applicable is true. Default 3.</t>
+          <t>Required. Currency of the invoice.</t>
         </is>
       </c>
       <c r="O3" s="3" t="inlineStr">
         <is>
-          <t>Required. Currency of the invoice.</t>
+          <t>Required. PEN per USD rate at transaction date. NUMERIC(10,4).</t>
         </is>
       </c>
       <c r="P3" s="3" t="inlineStr">
         <is>
-          <t>Required. PEN per USD rate at transaction date. NUMERIC(10,4).</t>
+          <t>Optional. Document reference linking to SharePoint file.</t>
         </is>
       </c>
       <c r="Q3" s="3" t="inlineStr">
         <is>
-          <t>Optional. Document reference linking to SharePoint file.</t>
+          <t>Required. Manually set to true once confirmed that client paid retención to SUNAT. BOOLEAN. Default false.</t>
         </is>
       </c>
       <c r="R3" s="3" t="inlineStr">
-        <is>
-          <t>Required. True when invoicing a partner company for settlement. BOOLEAN. Default false.</t>
-        </is>
-      </c>
-      <c r="S3" s="3" t="inlineStr">
-        <is>
-          <t>Required. Manually set to true once confirmed that client paid retención to SUNAT. BOOLEAN. Default false.</t>
-        </is>
-      </c>
-      <c r="T3" s="3" t="inlineStr">
         <is>
           <t>Optional. Free text notes.</t>
         </is>
@@ -814,71 +782,61 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Lookup → bank_accounts.bank_name</t>
+          <t>Lookup → bank_accounts.label</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Lookup → bank_accounts.account_number_last4</t>
+          <t>Lookup → entities.document_number</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Lookup → entities.document_number</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
           <t>Lookup → partner_companies.name</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr"/>
-      <c r="G4" s="4" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr"/>
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>factura | boleta | recibo_por_honorarios</t>
         </is>
       </c>
+      <c r="G4" s="4" t="inlineStr"/>
       <c r="H4" s="4" t="inlineStr"/>
       <c r="I4" s="4" t="inlineStr"/>
-      <c r="J4" s="4" t="inlineStr"/>
+      <c r="J4" s="4" t="inlineStr">
+        <is>
+          <t>Usually 18</t>
+        </is>
+      </c>
       <c r="K4" s="4" t="inlineStr">
         <is>
-          <t>Usually 18</t>
+          <t>Varies by service type</t>
         </is>
       </c>
       <c r="L4" s="4" t="inlineStr">
         <is>
-          <t>Varies by service type</t>
+          <t>true | false</t>
         </is>
       </c>
       <c r="M4" s="4" t="inlineStr">
         <is>
+          <t>Usually 3 (if applicable)</t>
+        </is>
+      </c>
+      <c r="N4" s="4" t="inlineStr">
+        <is>
+          <t>USD | PEN</t>
+        </is>
+      </c>
+      <c r="O4" s="4" t="inlineStr"/>
+      <c r="P4" s="4" t="inlineStr"/>
+      <c r="Q4" s="4" t="inlineStr">
+        <is>
           <t>true | false</t>
         </is>
       </c>
-      <c r="N4" s="4" t="inlineStr">
-        <is>
-          <t>Usually 3 (if applicable)</t>
-        </is>
-      </c>
-      <c r="O4" s="4" t="inlineStr">
-        <is>
-          <t>USD | PEN</t>
-        </is>
-      </c>
-      <c r="P4" s="4" t="inlineStr"/>
-      <c r="Q4" s="4" t="inlineStr"/>
-      <c r="R4" s="4" t="inlineStr">
-        <is>
-          <t>true | false</t>
-        </is>
-      </c>
-      <c r="S4" s="4" t="inlineStr">
-        <is>
-          <t>true | false</t>
-        </is>
-      </c>
-      <c r="T4" s="4" t="inlineStr"/>
+      <c r="R4" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>